<commit_message>
segments generating changed, hotel option added, no more midnight dependent. Timesheet template improved and formatted
</commit_message>
<xml_diff>
--- a/config/timesheet_template.xlsx
+++ b/config/timesheet_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petr/Documents/profi/expenses/01/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petr/code/travelrep/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A9D00B-9A4C-E54A-A72B-C003D166206E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13CA3C41-651F-B44C-A646-98F11D32802D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="32660" yWindow="3680" windowWidth="35140" windowHeight="13760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
   <si>
     <t>Date</t>
   </si>
@@ -98,9 +98,6 @@
     <t xml:space="preserve">R&amp;D % = </t>
   </si>
   <si>
-    <t>Travel home</t>
-  </si>
-  <si>
     <t>Date:</t>
   </si>
   <si>
@@ -110,15 +107,6 @@
     <t>XXXXX</t>
   </si>
   <si>
-    <t>% of RD- percent of minutes meeting</t>
-  </si>
-  <si>
-    <t>COunt all the minutes spent: Overall % r&amp;d</t>
-  </si>
-  <si>
-    <t>to be used for travel there and home</t>
-  </si>
-  <si>
     <t>xx</t>
   </si>
   <si>
@@ -126,36 +114,6 @@
   </si>
   <si>
     <t>XXX</t>
-  </si>
-  <si>
-    <t>x</t>
-  </si>
-  <si>
-    <t>Hutchinson PL - project Hutchinson PL</t>
-  </si>
-  <si>
-    <t>PASS PL - project PASS PL</t>
-  </si>
-  <si>
-    <t>Trave; there</t>
-  </si>
-  <si>
-    <t>Travel or meeting</t>
-  </si>
-  <si>
-    <t>each</t>
-  </si>
-  <si>
-    <t>day</t>
-  </si>
-  <si>
-    <t>travel or meeting</t>
-  </si>
-  <si>
-    <t>xxxx</t>
-  </si>
-  <si>
-    <t>xxx</t>
   </si>
 </sst>
 </file>
@@ -298,7 +256,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -362,12 +320,6 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -817,10 +769,10 @@
     </row>
     <row r="5" spans="1:8" ht="18" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -851,7 +803,7 @@
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -864,11 +816,11 @@
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="10"/>
-      <c r="F8" s="37" t="s">
+      <c r="F8" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="37"/>
-      <c r="H8" s="37"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="35"/>
     </row>
     <row r="9" spans="1:8" ht="57" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
@@ -898,243 +850,201 @@
     </row>
     <row r="10" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="22"/>
-      <c r="B10" s="23" t="s">
-        <v>33</v>
-      </c>
+      <c r="B10" s="23"/>
       <c r="C10" s="24"/>
       <c r="D10" s="24"/>
-      <c r="E10" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="G10" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="H10" s="21" t="s">
-        <v>30</v>
-      </c>
+      <c r="E10" s="31"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="21"/>
     </row>
     <row r="11" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="22"/>
-      <c r="B11" s="23" t="s">
-        <v>20</v>
-      </c>
+      <c r="B11" s="23"/>
       <c r="C11" s="24"/>
       <c r="D11" s="24"/>
-      <c r="E11" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="G11" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="H11" s="21" t="s">
-        <v>30</v>
-      </c>
+      <c r="E11" s="31"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="21"/>
     </row>
     <row r="12" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="22"/>
       <c r="B12" s="23"/>
       <c r="C12" s="24"/>
       <c r="D12" s="24"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="32"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="30"/>
       <c r="G12" s="25"/>
       <c r="H12" s="21"/>
     </row>
     <row r="13" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="22"/>
-      <c r="B13" s="21"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="32"/>
+      <c r="B13" s="23"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="30"/>
       <c r="G13" s="25"/>
       <c r="H13" s="21"/>
     </row>
     <row r="14" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="22" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="32"/>
+      <c r="A14" s="22"/>
+      <c r="B14" s="23"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="30"/>
       <c r="G14" s="25"/>
       <c r="H14" s="21"/>
     </row>
     <row r="15" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="32"/>
+      <c r="A15" s="22"/>
+      <c r="B15" s="23"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="30"/>
       <c r="G15" s="25"/>
-      <c r="H15" s="21" t="s">
-        <v>30</v>
-      </c>
+      <c r="H15" s="21"/>
     </row>
     <row r="16" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="22"/>
-      <c r="B16" s="21"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="32"/>
+      <c r="B16" s="23"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="30"/>
       <c r="G16" s="25"/>
       <c r="H16" s="21"/>
     </row>
     <row r="17" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="22"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="32"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="30"/>
       <c r="G17" s="25"/>
       <c r="H17" s="21"/>
     </row>
     <row r="18" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="22"/>
-      <c r="B18" s="21"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="32"/>
+      <c r="B18" s="23"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="30"/>
       <c r="G18" s="25"/>
-      <c r="H18" s="21" t="s">
-        <v>30</v>
-      </c>
+      <c r="H18" s="21"/>
     </row>
     <row r="19" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="22"/>
-      <c r="B19" s="21"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="32"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="30"/>
       <c r="G19" s="25"/>
       <c r="H19" s="21"/>
     </row>
     <row r="20" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="22"/>
-      <c r="B20" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="32"/>
+      <c r="B20" s="23"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="30"/>
       <c r="G20" s="25"/>
       <c r="H20" s="21"/>
     </row>
     <row r="21" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="22"/>
-      <c r="B21" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="32"/>
+      <c r="B21" s="23"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="30"/>
       <c r="G21" s="25"/>
       <c r="H21" s="21"/>
     </row>
     <row r="22" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="22"/>
       <c r="B22" s="23"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="27"/>
-      <c r="F22" s="32"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="30"/>
       <c r="G22" s="25"/>
       <c r="H22" s="21"/>
     </row>
     <row r="23" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="22"/>
       <c r="B23" s="23"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="27"/>
-      <c r="F23" s="32"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="31"/>
+      <c r="F23" s="30"/>
       <c r="G23" s="25"/>
       <c r="H23" s="21"/>
     </row>
     <row r="24" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="22"/>
       <c r="B24" s="23"/>
-      <c r="C24" s="28"/>
-      <c r="D24" s="28"/>
-      <c r="E24" s="27"/>
-      <c r="F24" s="32"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="30"/>
       <c r="G24" s="25"/>
       <c r="H24" s="21"/>
     </row>
     <row r="25" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="22"/>
-      <c r="B25" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="C25" s="28"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="27"/>
-      <c r="F25" s="32"/>
+      <c r="B25" s="23"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="31"/>
+      <c r="F25" s="30"/>
       <c r="G25" s="25"/>
       <c r="H25" s="21"/>
     </row>
     <row r="26" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="22"/>
-      <c r="B26" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="C26" s="28"/>
-      <c r="D26" s="28"/>
-      <c r="E26" s="27"/>
-      <c r="F26" s="32"/>
+      <c r="B26" s="23"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="30"/>
       <c r="G26" s="25"/>
       <c r="H26" s="21"/>
     </row>
     <row r="27" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="22"/>
-      <c r="B27" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="C27" s="28"/>
-      <c r="D27" s="28"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="32"/>
+      <c r="B27" s="23"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="30"/>
       <c r="G27" s="14"/>
       <c r="H27" s="21"/>
     </row>
     <row r="28" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="22"/>
       <c r="B28" s="23"/>
-      <c r="C28" s="28"/>
-      <c r="D28" s="28"/>
-      <c r="E28" s="27"/>
-      <c r="F28" s="32"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="30"/>
       <c r="G28" s="14"/>
       <c r="H28" s="21"/>
     </row>
     <row r="29" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="22"/>
       <c r="B29" s="23"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="27"/>
-      <c r="F29" s="32"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="30"/>
       <c r="G29" s="14"/>
       <c r="H29" s="21"/>
     </row>
@@ -1144,23 +1054,23 @@
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="26"/>
-      <c r="F30" s="32"/>
+      <c r="F30" s="30"/>
       <c r="G30" s="14"/>
       <c r="H30" s="20"/>
     </row>
     <row r="31" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
-      <c r="B31" s="30" t="s">
+      <c r="B31" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C31" s="31"/>
+      <c r="C31" s="29"/>
       <c r="D31" s="2"/>
       <c r="E31" s="26"/>
-      <c r="F31" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="G31" s="29" t="s">
-        <v>27</v>
+      <c r="F31" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="G31" s="27" t="s">
+        <v>23</v>
       </c>
       <c r="H31" s="20"/>
     </row>
@@ -1183,12 +1093,12 @@
         <v>3</v>
       </c>
       <c r="F33" s="15" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G33" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="H33" s="34">
+        <v>25</v>
+      </c>
+      <c r="H33" s="32">
         <f>SUM(H10:H32)</f>
         <v>0</v>
       </c>
@@ -1199,11 +1109,11 @@
       <c r="C34" s="16"/>
       <c r="D34" s="10"/>
       <c r="E34" s="16"/>
-      <c r="F34" s="36" t="s">
+      <c r="F34" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="G34" s="36"/>
-      <c r="H34" s="35">
+      <c r="G34" s="34"/>
+      <c r="H34" s="33">
         <v>0.16</v>
       </c>
     </row>
@@ -1215,11 +1125,11 @@
       <c r="C35" s="10"/>
       <c r="D35" s="10"/>
       <c r="E35" s="10"/>
-      <c r="F35" s="36" t="s">
+      <c r="F35" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="G35" s="36"/>
-      <c r="H35" s="35">
+      <c r="G35" s="34"/>
+      <c r="H35" s="33">
         <f>H33*H34</f>
         <v>0</v>
       </c>

</xml_diff>